<commit_message>
Revert cleanup commit and restore team context pages
</commit_message>
<xml_diff>
--- a/data/2FEB_25_26/teams_25_26_2FEB.xlsx
+++ b/data/2FEB_25_26/teams_25_26_2FEB.xlsx
@@ -852,244 +852,244 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9392530869325559</v>
+        <v>0.9071826934173232</v>
       </c>
       <c r="D2" t="n">
-        <v>0.916965931824948</v>
+        <v>0.9137151890637706</v>
       </c>
       <c r="E2" t="n">
-        <v>107.7631782770694</v>
+        <v>104.631171924052</v>
       </c>
       <c r="F2" t="n">
-        <v>101.0345280578546</v>
+        <v>100.3654189735666</v>
       </c>
       <c r="G2" t="n">
-        <v>6.728650219214833</v>
+        <v>4.265752950485385</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3419454531657249</v>
+        <v>0.3433172203488318</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7570842754136318</v>
+        <v>0.7626580697912553</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5431698241552574</v>
+        <v>0.5423170704790934</v>
       </c>
       <c r="K2" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L2" t="n">
-        <v>2099</v>
+        <v>1816</v>
       </c>
       <c r="M2" t="n">
-        <v>473</v>
+        <v>402</v>
       </c>
       <c r="N2" t="n">
-        <v>909</v>
+        <v>804</v>
       </c>
       <c r="O2" t="n">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="P2" t="n">
-        <v>757</v>
+        <v>674</v>
       </c>
       <c r="Q2" t="n">
-        <v>406</v>
+        <v>367</v>
       </c>
       <c r="R2" t="n">
-        <v>560</v>
+        <v>514</v>
       </c>
       <c r="S2" t="n">
-        <v>291</v>
+        <v>267</v>
       </c>
       <c r="T2" t="n">
-        <v>612</v>
+        <v>542</v>
       </c>
       <c r="U2" t="n">
-        <v>353</v>
+        <v>301</v>
       </c>
       <c r="V2" t="n">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="W2" t="n">
-        <v>332</v>
+        <v>302</v>
       </c>
       <c r="X2" t="n">
-        <v>608</v>
+        <v>540</v>
       </c>
       <c r="Y2" t="n">
-        <v>553</v>
+        <v>500</v>
       </c>
       <c r="Z2" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="AA2" t="n">
-        <v>1968</v>
+        <v>1734</v>
       </c>
       <c r="AB2" t="n">
-        <v>2244.4</v>
+        <v>2006.16</v>
       </c>
       <c r="AC2" t="n">
-        <v>1953.4</v>
+        <v>1739.16</v>
       </c>
       <c r="AD2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE2" t="n">
-        <v>2600</v>
+        <v>2400</v>
       </c>
       <c r="AF2" t="n">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="AG2" t="n">
-        <v>444</v>
+        <v>410</v>
       </c>
       <c r="AH2" t="n">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="AI2" t="n">
-        <v>385</v>
+        <v>361</v>
       </c>
       <c r="AJ2" t="n">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="AK2" t="n">
-        <v>276</v>
+        <v>263</v>
       </c>
       <c r="AL2" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="AM2" t="n">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="AN2" t="n">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="AO2" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="AP2" t="n">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="AQ2" t="n">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="AR2" t="n">
-        <v>275</v>
+        <v>257</v>
       </c>
       <c r="AS2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AT2" t="n">
-        <v>1114.44</v>
+        <v>1040.72</v>
       </c>
       <c r="AU2" t="n">
-        <v>975.4400000000001</v>
+        <v>908.72</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.877614405034956</v>
+        <v>0.8591862692273698</v>
       </c>
       <c r="AW2" t="n">
-        <v>0.9103141686203858</v>
+        <v>0.9075009611934358</v>
       </c>
       <c r="AX2" t="n">
-        <v>100.3288522059469</v>
+        <v>98.57268341495565</v>
       </c>
       <c r="AY2" t="n">
-        <v>100.7602111333452</v>
+        <v>100.2218610115402</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-0.4313589273983627</v>
+        <v>-1.649177596584586</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.3238647880965319</v>
+        <v>0.3275201871045761</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.7501196426315435</v>
+        <v>0.7553379461841722</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.5252537884174946</v>
+        <v>0.5266272766335723</v>
       </c>
       <c r="BD2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BE2" t="n">
-        <v>2625</v>
+        <v>2225</v>
       </c>
       <c r="BF2" t="n">
-        <v>257</v>
+        <v>209</v>
       </c>
       <c r="BG2" t="n">
-        <v>465</v>
+        <v>394</v>
       </c>
       <c r="BH2" t="n">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="BI2" t="n">
-        <v>372</v>
+        <v>313</v>
       </c>
       <c r="BJ2" t="n">
-        <v>215</v>
+        <v>187</v>
       </c>
       <c r="BK2" t="n">
-        <v>284</v>
+        <v>251</v>
       </c>
       <c r="BL2" t="n">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="BM2" t="n">
-        <v>310</v>
+        <v>262</v>
       </c>
       <c r="BN2" t="n">
-        <v>197</v>
+        <v>160</v>
       </c>
       <c r="BO2" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="BP2" t="n">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="BQ2" t="n">
-        <v>306</v>
+        <v>262</v>
       </c>
       <c r="BR2" t="n">
-        <v>278</v>
+        <v>243</v>
       </c>
       <c r="BS2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BT2" t="n">
-        <v>1129.96</v>
+        <v>965.4400000000001</v>
       </c>
       <c r="BU2" t="n">
-        <v>977.96</v>
+        <v>830.4400000000001</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.000891768830156</v>
+        <v>0.9595424288972723</v>
       </c>
       <c r="BW2" t="n">
-        <v>0.9236176950295103</v>
+        <v>0.9204943467404992</v>
       </c>
       <c r="BX2" t="n">
-        <v>115.1975043481919</v>
+        <v>111.2404321157935</v>
       </c>
       <c r="BY2" t="n">
-        <v>101.3088449823639</v>
+        <v>100.5220276594136</v>
       </c>
       <c r="BZ2" t="n">
-        <v>13.88865936582803</v>
+        <v>10.7184044563799</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.3600261182349179</v>
+        <v>0.3605503475243836</v>
       </c>
       <c r="CB2" t="n">
-        <v>0.7640489081957198</v>
+        <v>0.7706436591808004</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.5610858598930202</v>
+        <v>0.5594332092196618</v>
       </c>
       <c r="CD2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -1104,244 +1104,244 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9500327614568331</v>
+        <v>0.9368424371285909</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9053845880874861</v>
+        <v>0.906282227956188</v>
       </c>
       <c r="E3" t="n">
-        <v>105.7308988642809</v>
+        <v>104.8323947497282</v>
       </c>
       <c r="F3" t="n">
-        <v>101.281866828337</v>
+        <v>100.9059924914148</v>
       </c>
       <c r="G3" t="n">
-        <v>4.44903203594398</v>
+        <v>3.926402258313354</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2703448107574296</v>
+        <v>0.2784957331001028</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7307218761813891</v>
+        <v>0.7382991398985331</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5101275234043477</v>
+        <v>0.5135078610691944</v>
       </c>
       <c r="K3" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L3" t="n">
-        <v>2064</v>
+        <v>1809</v>
       </c>
       <c r="M3" t="n">
-        <v>539</v>
+        <v>481</v>
       </c>
       <c r="N3" t="n">
-        <v>998</v>
+        <v>891</v>
       </c>
       <c r="O3" t="n">
-        <v>198</v>
+        <v>171</v>
       </c>
       <c r="P3" t="n">
-        <v>602</v>
+        <v>546</v>
       </c>
       <c r="Q3" t="n">
-        <v>392</v>
+        <v>334</v>
       </c>
       <c r="R3" t="n">
-        <v>594</v>
+        <v>506</v>
       </c>
       <c r="S3" t="n">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="T3" t="n">
-        <v>638</v>
+        <v>561</v>
       </c>
       <c r="U3" t="n">
-        <v>384</v>
+        <v>325</v>
       </c>
       <c r="V3" t="n">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="W3" t="n">
-        <v>322</v>
+        <v>281</v>
       </c>
       <c r="X3" t="n">
-        <v>554</v>
+        <v>496</v>
       </c>
       <c r="Y3" t="n">
-        <v>558</v>
+        <v>486</v>
       </c>
       <c r="Z3" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="AA3" t="n">
-        <v>1997</v>
+        <v>1755</v>
       </c>
       <c r="AB3" t="n">
-        <v>2183.36</v>
+        <v>1940.64</v>
       </c>
       <c r="AC3" t="n">
-        <v>1954.36</v>
+        <v>1727.64</v>
       </c>
       <c r="AD3" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE3" t="n">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="AF3" t="n">
-        <v>268</v>
+        <v>228</v>
       </c>
       <c r="AG3" t="n">
-        <v>487</v>
+        <v>411</v>
       </c>
       <c r="AH3" t="n">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="AI3" t="n">
-        <v>300</v>
+        <v>264</v>
       </c>
       <c r="AJ3" t="n">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="AK3" t="n">
-        <v>277</v>
+        <v>232</v>
       </c>
       <c r="AL3" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="AM3" t="n">
-        <v>314</v>
+        <v>271</v>
       </c>
       <c r="AN3" t="n">
-        <v>186</v>
+        <v>144</v>
       </c>
       <c r="AO3" t="n">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AP3" t="n">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="AQ3" t="n">
-        <v>278</v>
+        <v>240</v>
       </c>
       <c r="AR3" t="n">
-        <v>270</v>
+        <v>228</v>
       </c>
       <c r="AS3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AT3" t="n">
-        <v>1071.88</v>
+        <v>910.08</v>
       </c>
       <c r="AU3" t="n">
-        <v>960.88</v>
+        <v>812.08</v>
       </c>
       <c r="AV3" t="n">
-        <v>0.969155424877412</v>
+        <v>0.9564255196558107</v>
       </c>
       <c r="AW3" t="n">
-        <v>0.8714974560799997</v>
+        <v>0.866462551669141</v>
       </c>
       <c r="AX3" t="n">
-        <v>107.6256025405429</v>
+        <v>106.6297744738392</v>
       </c>
       <c r="AY3" t="n">
-        <v>98.50338342831387</v>
+        <v>96.79115989726751</v>
       </c>
       <c r="AZ3" t="n">
-        <v>9.122219112228983</v>
+        <v>9.838614576571722</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.2687794873988426</v>
+        <v>0.2723245561631044</v>
       </c>
       <c r="BB3" t="n">
-        <v>0.713559734915546</v>
+        <v>0.7371261809865678</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.502171214484582</v>
+        <v>0.5139741803979997</v>
       </c>
       <c r="BD3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="BE3" t="n">
-        <v>2625</v>
+        <v>2425</v>
       </c>
       <c r="BF3" t="n">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="BG3" t="n">
-        <v>511</v>
+        <v>480</v>
       </c>
       <c r="BH3" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="BI3" t="n">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="BJ3" t="n">
-        <v>212</v>
+        <v>182</v>
       </c>
       <c r="BK3" t="n">
-        <v>317</v>
+        <v>274</v>
       </c>
       <c r="BL3" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="BM3" t="n">
-        <v>324</v>
+        <v>290</v>
       </c>
       <c r="BN3" t="n">
-        <v>198</v>
+        <v>181</v>
       </c>
       <c r="BO3" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="BP3" t="n">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="BQ3" t="n">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="BR3" t="n">
-        <v>288</v>
+        <v>258</v>
       </c>
       <c r="BS3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="BT3" t="n">
-        <v>1111.48</v>
+        <v>1030.56</v>
       </c>
       <c r="BU3" t="n">
-        <v>993.48</v>
+        <v>915.5600000000001</v>
       </c>
       <c r="BV3" t="n">
-        <v>0.9309100980362542</v>
+        <v>0.9188912781453059</v>
       </c>
       <c r="BW3" t="n">
-        <v>0.9392717200949725</v>
+        <v>0.942783597885981</v>
       </c>
       <c r="BX3" t="n">
-        <v>103.836195188019</v>
+        <v>103.184796669293</v>
       </c>
       <c r="BY3" t="n">
-        <v>104.06035022836</v>
+        <v>104.6779223693832</v>
       </c>
       <c r="BZ3" t="n">
-        <v>-0.2241550403410217</v>
+        <v>-1.49312570009015</v>
       </c>
       <c r="CA3" t="n">
-        <v>0.2719101341160164</v>
+        <v>0.2841526452923511</v>
       </c>
       <c r="CB3" t="n">
-        <v>0.7478840174472319</v>
+        <v>0.7393743522345012</v>
       </c>
       <c r="CC3" t="n">
-        <v>0.5180838323241135</v>
+        <v>0.5130804016844562</v>
       </c>
       <c r="CD3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -1356,244 +1356,244 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9674707923982999</v>
+        <v>0.9802706716177139</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8848949565287919</v>
+        <v>0.8810225151559815</v>
       </c>
       <c r="E4" t="n">
-        <v>108.4379226657104</v>
+        <v>109.1754572015646</v>
       </c>
       <c r="F4" t="n">
-        <v>101.5899314586172</v>
+        <v>101.3240938581334</v>
       </c>
       <c r="G4" t="n">
-        <v>6.847991207093241</v>
+        <v>7.851363343431153</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2873329318053095</v>
+        <v>0.2811810972150894</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6957587239933678</v>
+        <v>0.6952277957193879</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5077443188030457</v>
+        <v>0.5092691397287213</v>
       </c>
       <c r="K4" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L4" t="n">
-        <v>2135</v>
+        <v>1902</v>
       </c>
       <c r="M4" t="n">
-        <v>507</v>
+        <v>450</v>
       </c>
       <c r="N4" t="n">
-        <v>960</v>
+        <v>847</v>
       </c>
       <c r="O4" t="n">
-        <v>230</v>
+        <v>208</v>
       </c>
       <c r="P4" t="n">
-        <v>662</v>
+        <v>572</v>
       </c>
       <c r="Q4" t="n">
-        <v>431</v>
+        <v>378</v>
       </c>
       <c r="R4" t="n">
-        <v>613</v>
+        <v>532</v>
       </c>
       <c r="S4" t="n">
-        <v>243</v>
+        <v>201</v>
       </c>
       <c r="T4" t="n">
-        <v>670</v>
+        <v>601</v>
       </c>
       <c r="U4" t="n">
-        <v>352</v>
+        <v>331</v>
       </c>
       <c r="V4" t="n">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="W4" t="n">
-        <v>319</v>
+        <v>291</v>
       </c>
       <c r="X4" t="n">
-        <v>546</v>
+        <v>480</v>
       </c>
       <c r="Y4" t="n">
-        <v>568</v>
+        <v>494</v>
       </c>
       <c r="Z4" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="AA4" t="n">
-        <v>2012</v>
+        <v>1782</v>
       </c>
       <c r="AB4" t="n">
-        <v>2210.72</v>
+        <v>1944.08</v>
       </c>
       <c r="AC4" t="n">
-        <v>1967.72</v>
+        <v>1743.08</v>
       </c>
       <c r="AD4" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE4" t="n">
-        <v>2600</v>
+        <v>2400</v>
       </c>
       <c r="AF4" t="n">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="AG4" t="n">
-        <v>474</v>
+        <v>438</v>
       </c>
       <c r="AH4" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="AI4" t="n">
-        <v>329</v>
+        <v>300</v>
       </c>
       <c r="AJ4" t="n">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="AK4" t="n">
-        <v>290</v>
+        <v>266</v>
       </c>
       <c r="AL4" t="n">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="AM4" t="n">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="AN4" t="n">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="AO4" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="AP4" t="n">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="AQ4" t="n">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="AR4" t="n">
-        <v>274</v>
+        <v>250</v>
       </c>
       <c r="AS4" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AT4" t="n">
-        <v>1084.6</v>
+        <v>999.04</v>
       </c>
       <c r="AU4" t="n">
-        <v>980.6</v>
+        <v>908.04</v>
       </c>
       <c r="AV4" t="n">
-        <v>1.033763634595694</v>
+        <v>1.044914500046846</v>
       </c>
       <c r="AW4" t="n">
-        <v>0.8908992845072363</v>
+        <v>0.894726290377807</v>
       </c>
       <c r="AX4" t="n">
-        <v>114.2713961260163</v>
+        <v>114.9507563140259</v>
       </c>
       <c r="AY4" t="n">
-        <v>103.6346673328864</v>
+        <v>103.6810050586753</v>
       </c>
       <c r="AZ4" t="n">
-        <v>10.6367287931299</v>
+        <v>11.26975125535062</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.2763270102965038</v>
+        <v>0.2722709278212124</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.6638306887610229</v>
+        <v>0.6750322657656179</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.495346754770606</v>
+        <v>0.5017157410915799</v>
       </c>
       <c r="BD4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BE4" t="n">
-        <v>2625</v>
+        <v>2225</v>
       </c>
       <c r="BF4" t="n">
-        <v>249</v>
+        <v>208</v>
       </c>
       <c r="BG4" t="n">
-        <v>486</v>
+        <v>409</v>
       </c>
       <c r="BH4" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="BI4" t="n">
-        <v>333</v>
+        <v>272</v>
       </c>
       <c r="BJ4" t="n">
-        <v>220</v>
+        <v>182</v>
       </c>
       <c r="BK4" t="n">
-        <v>323</v>
+        <v>266</v>
       </c>
       <c r="BL4" t="n">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="BM4" t="n">
-        <v>350</v>
+        <v>299</v>
       </c>
       <c r="BN4" t="n">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="BO4" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="BP4" t="n">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="BQ4" t="n">
-        <v>273</v>
+        <v>228</v>
       </c>
       <c r="BR4" t="n">
-        <v>294</v>
+        <v>244</v>
       </c>
       <c r="BS4" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="BT4" t="n">
-        <v>1126.12</v>
+        <v>945.04</v>
       </c>
       <c r="BU4" t="n">
-        <v>987.12</v>
+        <v>835.04</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.9011779502009063</v>
+        <v>0.9097501315132054</v>
       </c>
       <c r="BW4" t="n">
-        <v>0.8788906285503481</v>
+        <v>0.8660729421867178</v>
       </c>
       <c r="BX4" t="n">
-        <v>102.6044492054045</v>
+        <v>102.8751308970613</v>
       </c>
       <c r="BY4" t="n">
-        <v>99.54519558434789</v>
+        <v>98.75291800299679</v>
       </c>
       <c r="BZ4" t="n">
-        <v>3.059253621056574</v>
+        <v>4.122212894064458</v>
       </c>
       <c r="CA4" t="n">
-        <v>0.298338853314115</v>
+        <v>0.2909012820084095</v>
       </c>
       <c r="CB4" t="n">
-        <v>0.7276867592257126</v>
+        <v>0.7172592829416824</v>
       </c>
       <c r="CC4" t="n">
-        <v>0.5201418828354855</v>
+        <v>0.5175092109692394</v>
       </c>
       <c r="CD4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -1608,244 +1608,244 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8575797836063584</v>
+        <v>0.8565378540291038</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9643797201496689</v>
+        <v>0.9693443419295926</v>
       </c>
       <c r="E5" t="n">
-        <v>95.98195606809885</v>
+        <v>96.05032997385878</v>
       </c>
       <c r="F5" t="n">
-        <v>112.1181890457704</v>
+        <v>112.5908367765532</v>
       </c>
       <c r="G5" t="n">
-        <v>-16.13623297767151</v>
+        <v>-16.54050680269442</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2670976649304634</v>
+        <v>0.2712354587312309</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6334981930449425</v>
+        <v>0.6316244217642256</v>
       </c>
       <c r="J5" t="n">
-        <v>0.4496051100222618</v>
+        <v>0.4496466131288217</v>
       </c>
       <c r="K5" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L5" t="n">
-        <v>1938</v>
+        <v>1718</v>
       </c>
       <c r="M5" t="n">
-        <v>472</v>
+        <v>412</v>
       </c>
       <c r="N5" t="n">
-        <v>987</v>
+        <v>869</v>
       </c>
       <c r="O5" t="n">
+        <v>194</v>
+      </c>
+      <c r="P5" t="n">
+        <v>602</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>312</v>
+      </c>
+      <c r="R5" t="n">
+        <v>436</v>
+      </c>
+      <c r="S5" t="n">
+        <v>218</v>
+      </c>
+      <c r="T5" t="n">
+        <v>497</v>
+      </c>
+      <c r="U5" t="n">
+        <v>277</v>
+      </c>
+      <c r="V5" t="n">
+        <v>165</v>
+      </c>
+      <c r="W5" t="n">
+        <v>342</v>
+      </c>
+      <c r="X5" t="n">
+        <v>522</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>457</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>54</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>2014</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>2004.84</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1786.84</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>2425</v>
+      </c>
+      <c r="AF5" t="n">
         <v>212</v>
       </c>
-      <c r="P5" t="n">
-        <v>662</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>358</v>
-      </c>
-      <c r="R5" t="n">
-        <v>509</v>
-      </c>
-      <c r="S5" t="n">
-        <v>242</v>
-      </c>
-      <c r="T5" t="n">
-        <v>568</v>
-      </c>
-      <c r="U5" t="n">
-        <v>326</v>
-      </c>
-      <c r="V5" t="n">
-        <v>185</v>
-      </c>
-      <c r="W5" t="n">
-        <v>386</v>
-      </c>
-      <c r="X5" t="n">
-        <v>583</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>522</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>60</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>2260</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>2258.96</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>2016.96</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>26</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>2625</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>236</v>
-      </c>
       <c r="AG5" t="n">
-        <v>489</v>
+        <v>446</v>
       </c>
       <c r="AH5" t="n">
         <v>114</v>
       </c>
       <c r="AI5" t="n">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="AJ5" t="n">
-        <v>202</v>
+        <v>182</v>
       </c>
       <c r="AK5" t="n">
-        <v>275</v>
+        <v>248</v>
       </c>
       <c r="AL5" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="AM5" t="n">
-        <v>282</v>
+        <v>259</v>
       </c>
       <c r="AN5" t="n">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="AO5" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="AP5" t="n">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="AQ5" t="n">
-        <v>292</v>
+        <v>271</v>
       </c>
       <c r="AR5" t="n">
-        <v>261</v>
+        <v>237</v>
       </c>
       <c r="AS5" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="AT5" t="n">
-        <v>1125</v>
+        <v>1044.12</v>
       </c>
       <c r="AU5" t="n">
-        <v>1021</v>
+        <v>946.12</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.9022859123995398</v>
+        <v>0.9074137608528811</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.9829465747987606</v>
+        <v>0.983253566631069</v>
       </c>
       <c r="AX5" t="n">
-        <v>99.51127526698328</v>
+        <v>100.2362177215681</v>
       </c>
       <c r="AY5" t="n">
-        <v>114.0532515974638</v>
+        <v>114.334598952808</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-14.54197633048055</v>
+        <v>-14.09838123123997</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.2384259290338632</v>
+        <v>0.2431432413018366</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.6324304294033087</v>
+        <v>0.6270521571061097</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.4367255802038411</v>
+        <v>0.4365032169379996</v>
       </c>
       <c r="BD5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BE5" t="n">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="BF5" t="n">
-        <v>236</v>
+        <v>200</v>
       </c>
       <c r="BG5" t="n">
-        <v>498</v>
+        <v>423</v>
       </c>
       <c r="BH5" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="BI5" t="n">
-        <v>341</v>
+        <v>294</v>
       </c>
       <c r="BJ5" t="n">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="BK5" t="n">
-        <v>234</v>
+        <v>188</v>
       </c>
       <c r="BL5" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="BM5" t="n">
-        <v>286</v>
+        <v>238</v>
       </c>
       <c r="BN5" t="n">
-        <v>152</v>
+        <v>120</v>
       </c>
       <c r="BO5" t="n">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="BP5" t="n">
-        <v>192</v>
+        <v>161</v>
       </c>
       <c r="BQ5" t="n">
-        <v>291</v>
+        <v>251</v>
       </c>
       <c r="BR5" t="n">
-        <v>261</v>
+        <v>220</v>
       </c>
       <c r="BS5" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="BT5" t="n">
-        <v>1133.96</v>
+        <v>960.72</v>
       </c>
       <c r="BU5" t="n">
-        <v>995.96</v>
+        <v>840.72</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.812873654813177</v>
+        <v>0.8010368647668014</v>
       </c>
       <c r="BW5" t="n">
-        <v>0.9458128655005774</v>
+        <v>0.9541706422552551</v>
       </c>
       <c r="BX5" t="n">
-        <v>92.45263686921443</v>
+        <v>91.48390697635776</v>
       </c>
       <c r="BY5" t="n">
-        <v>110.1831264940769</v>
+        <v>110.6885507660934</v>
       </c>
       <c r="BZ5" t="n">
-        <v>-17.73048962486246</v>
+        <v>-19.20464378973562</v>
       </c>
       <c r="CA5" t="n">
-        <v>0.2957694008270637</v>
+        <v>0.301881514108752</v>
       </c>
       <c r="CB5" t="n">
-        <v>0.6345659566865767</v>
+        <v>0.6366123468458067</v>
       </c>
       <c r="CC5" t="n">
-        <v>0.4624846398406824</v>
+        <v>0.4639848635188094</v>
       </c>
       <c r="CD5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -1860,244 +1860,244 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9124083077020527</v>
+        <v>0.9184225819425451</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8529228177756895</v>
+        <v>0.8595846726535051</v>
       </c>
       <c r="E6" t="n">
-        <v>102.6298065817949</v>
+        <v>103.1774419626771</v>
       </c>
       <c r="F6" t="n">
-        <v>97.47734296304385</v>
+        <v>98.00957171490018</v>
       </c>
       <c r="G6" t="n">
-        <v>5.152463618751072</v>
+        <v>5.167870247776921</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2818409191161311</v>
+        <v>0.2800523579632114</v>
       </c>
       <c r="I6" t="n">
-        <v>0.7062816771281473</v>
+        <v>0.7086790994084761</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5050318350355452</v>
+        <v>0.5049000473182583</v>
       </c>
       <c r="K6" t="n">
-        <v>5275</v>
+        <v>4675</v>
       </c>
       <c r="L6" t="n">
-        <v>2055</v>
+        <v>1839</v>
       </c>
       <c r="M6" t="n">
-        <v>498</v>
+        <v>453</v>
       </c>
       <c r="N6" t="n">
-        <v>954</v>
+        <v>856</v>
       </c>
       <c r="O6" t="n">
-        <v>208</v>
+        <v>183</v>
       </c>
       <c r="P6" t="n">
-        <v>658</v>
+        <v>585</v>
       </c>
       <c r="Q6" t="n">
-        <v>435</v>
+        <v>384</v>
       </c>
       <c r="R6" t="n">
-        <v>641</v>
+        <v>556</v>
       </c>
       <c r="S6" t="n">
-        <v>251</v>
+        <v>221</v>
       </c>
       <c r="T6" t="n">
-        <v>697</v>
+        <v>616</v>
       </c>
       <c r="U6" t="n">
-        <v>456</v>
+        <v>416</v>
       </c>
       <c r="V6" t="n">
-        <v>165</v>
+        <v>144</v>
       </c>
       <c r="W6" t="n">
-        <v>357</v>
+        <v>316</v>
       </c>
       <c r="X6" t="n">
-        <v>577</v>
+        <v>509</v>
       </c>
       <c r="Y6" t="n">
-        <v>597</v>
+        <v>528</v>
       </c>
       <c r="Z6" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="AA6" t="n">
-        <v>1961</v>
+        <v>1750</v>
       </c>
       <c r="AB6" t="n">
-        <v>2251.04</v>
+        <v>2001.64</v>
       </c>
       <c r="AC6" t="n">
-        <v>2000.04</v>
+        <v>1780.64</v>
       </c>
       <c r="AD6" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE6" t="n">
-        <v>2650</v>
+        <v>2450</v>
       </c>
       <c r="AF6" t="n">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="AG6" t="n">
-        <v>471</v>
+        <v>446</v>
       </c>
       <c r="AH6" t="n">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="AI6" t="n">
-        <v>322</v>
+        <v>291</v>
       </c>
       <c r="AJ6" t="n">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="AK6" t="n">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="AL6" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="AM6" t="n">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="AN6" t="n">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="AO6" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="AP6" t="n">
+        <v>169</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>265</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>272</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>18</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>1031.4</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>922.4</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0.8836888367761886</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0.9065455078874267</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>98.70234164655737</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>102.4826112269313</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>-3.780269580373916</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>0.2657710912961013</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>0.7075326379109587</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.4916391746841752</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>227</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>410</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>97</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>294</v>
+      </c>
+      <c r="BJ6" t="n">
         <v>182</v>
       </c>
-      <c r="AQ6" t="n">
-        <v>289</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>292</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>19</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>1110.08</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>995.08</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>0.8802389935186405</v>
-      </c>
-      <c r="AW6" t="n">
-        <v>0.8937649275811322</v>
-      </c>
-      <c r="AX6" t="n">
-        <v>98.09516350965399</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>101.0397794411298</v>
-      </c>
-      <c r="AZ6" t="n">
-        <v>-2.944615931475837</v>
-      </c>
-      <c r="BA6" t="n">
-        <v>0.2597502381194782</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>0.7080521053244013</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>0.4894120510287909</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>13</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>2625</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>265</v>
-      </c>
-      <c r="BG6" t="n">
-        <v>483</v>
-      </c>
-      <c r="BH6" t="n">
-        <v>109</v>
-      </c>
-      <c r="BI6" t="n">
-        <v>336</v>
-      </c>
-      <c r="BJ6" t="n">
-        <v>220</v>
-      </c>
       <c r="BK6" t="n">
-        <v>334</v>
+        <v>271</v>
       </c>
       <c r="BL6" t="n">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="BM6" t="n">
-        <v>376</v>
+        <v>320</v>
       </c>
       <c r="BN6" t="n">
-        <v>263</v>
+        <v>235</v>
       </c>
       <c r="BO6" t="n">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="BP6" t="n">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="BQ6" t="n">
-        <v>288</v>
+        <v>244</v>
       </c>
       <c r="BR6" t="n">
-        <v>305</v>
+        <v>256</v>
       </c>
       <c r="BS6" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="BT6" t="n">
-        <v>1140.96</v>
+        <v>970.24</v>
       </c>
       <c r="BU6" t="n">
-        <v>1004.96</v>
+        <v>858.24</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.9445776218854649</v>
+        <v>0.9563139403058429</v>
       </c>
       <c r="BW6" t="n">
-        <v>0.8120807079702469</v>
+        <v>0.8083546705801364</v>
       </c>
       <c r="BX6" t="n">
-        <v>107.1644496539359</v>
+        <v>108.0593695802622</v>
       </c>
       <c r="BY6" t="n">
-        <v>93.91490648495788</v>
+        <v>93.12989224722986</v>
       </c>
       <c r="BZ6" t="n">
-        <v>13.24954316897798</v>
+        <v>14.92947733303238</v>
       </c>
       <c r="CA6" t="n">
-        <v>0.3039316001127841</v>
+        <v>0.2956319216000589</v>
       </c>
       <c r="CB6" t="n">
-        <v>0.7045112489318933</v>
+        <v>0.7099297846784954</v>
       </c>
       <c r="CC6" t="n">
-        <v>0.5206516190422993</v>
+        <v>0.5193664538281668</v>
       </c>
       <c r="CD6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -2112,244 +2112,244 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9099260347198977</v>
+        <v>0.9051179369430532</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9164536409182822</v>
+        <v>0.9186644392943949</v>
       </c>
       <c r="E7" t="n">
-        <v>101.8883941489013</v>
+        <v>101.5641550028868</v>
       </c>
       <c r="F7" t="n">
-        <v>100.9477344635132</v>
+        <v>101.7766779529189</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9406596853880979</v>
+        <v>-0.2125229500320535</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2688618123165215</v>
+        <v>0.2728477564400011</v>
       </c>
       <c r="I7" t="n">
-        <v>0.7606278906477331</v>
+        <v>0.7488472747392706</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5041204554325289</v>
+        <v>0.5032690881283732</v>
       </c>
       <c r="K7" t="n">
-        <v>5225</v>
+        <v>4600</v>
       </c>
       <c r="L7" t="n">
-        <v>2030</v>
+        <v>1786</v>
       </c>
       <c r="M7" t="n">
-        <v>429</v>
+        <v>374</v>
       </c>
       <c r="N7" t="n">
-        <v>902</v>
+        <v>802</v>
       </c>
       <c r="O7" t="n">
+        <v>214</v>
+      </c>
+      <c r="P7" t="n">
+        <v>636</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>396</v>
+      </c>
+      <c r="R7" t="n">
+        <v>560</v>
+      </c>
+      <c r="S7" t="n">
+        <v>214</v>
+      </c>
+      <c r="T7" t="n">
+        <v>555</v>
+      </c>
+      <c r="U7" t="n">
+        <v>299</v>
+      </c>
+      <c r="V7" t="n">
+        <v>147</v>
+      </c>
+      <c r="W7" t="n">
+        <v>290</v>
+      </c>
+      <c r="X7" t="n">
+        <v>519</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>531</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1787</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1974.4</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1760.4</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>200</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>434</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>89</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>317</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>209</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>301</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>107</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>280</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>140</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>77</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>142</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>274</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>276</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>12</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>1025.44</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>918.4399999999999</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.8554146867260263</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.9517565461268437</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>95.430011340592</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>105.7521649474348</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>-10.32215360684274</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.2525017948458839</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>0.7398088666664293</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.4797812864746899</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>2200</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>174</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>368</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>125</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>319</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>187</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>259</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>107</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>275</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>159</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>70</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>148</v>
+      </c>
+      <c r="BQ7" t="n">
         <v>245</v>
       </c>
-      <c r="P7" t="n">
-        <v>730</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>437</v>
-      </c>
-      <c r="R7" t="n">
-        <v>614</v>
-      </c>
-      <c r="S7" t="n">
-        <v>238</v>
-      </c>
-      <c r="T7" t="n">
-        <v>628</v>
-      </c>
-      <c r="U7" t="n">
-        <v>341</v>
-      </c>
-      <c r="V7" t="n">
-        <v>172</v>
-      </c>
-      <c r="W7" t="n">
-        <v>330</v>
-      </c>
-      <c r="X7" t="n">
-        <v>590</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>591</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>28</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>2012</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>2232.16</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>1994.16</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>26</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>2600</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>216</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>465</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>100</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>354</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>219</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>316</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>113</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>301</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>151</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>84</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>151</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>305</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>296</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>14</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>1109.04</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>996.04</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>0.8586234944088604</v>
-      </c>
-      <c r="AW7" t="n">
-        <v>0.9612472684807505</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>95.52381697101436</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>106.2060735986114</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>-10.68225662759703</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>0.2446170413962005</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>0.7502081846151655</v>
-      </c>
-      <c r="BC7" t="n">
-        <v>0.4753269567458676</v>
-      </c>
-      <c r="BD7" t="n">
+      <c r="BR7" t="n">
+        <v>255</v>
+      </c>
+      <c r="BS7" t="n">
         <v>13</v>
       </c>
-      <c r="BE7" t="n">
-        <v>2625</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>213</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>437</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>145</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>376</v>
-      </c>
-      <c r="BJ7" t="n">
-        <v>218</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>298</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>125</v>
-      </c>
-      <c r="BM7" t="n">
-        <v>327</v>
-      </c>
-      <c r="BN7" t="n">
-        <v>190</v>
-      </c>
-      <c r="BO7" t="n">
-        <v>88</v>
-      </c>
-      <c r="BP7" t="n">
-        <v>179</v>
-      </c>
-      <c r="BQ7" t="n">
-        <v>285</v>
-      </c>
-      <c r="BR7" t="n">
-        <v>295</v>
-      </c>
-      <c r="BS7" t="n">
-        <v>14</v>
-      </c>
       <c r="BT7" t="n">
-        <v>1123.12</v>
+        <v>948.96</v>
       </c>
       <c r="BU7" t="n">
-        <v>998.12</v>
+        <v>841.96</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.9612285750309351</v>
+        <v>0.959339664452537</v>
       </c>
       <c r="BW7" t="n">
-        <v>0.8716600133558134</v>
+        <v>0.882563959113541</v>
       </c>
       <c r="BX7" t="n">
-        <v>108.2529713267882</v>
+        <v>108.2559480890266</v>
       </c>
       <c r="BY7" t="n">
-        <v>95.68939532841502</v>
+        <v>97.43978304981064</v>
       </c>
       <c r="BZ7" t="n">
-        <v>12.56357599837322</v>
+        <v>10.81616503921596</v>
       </c>
       <c r="CA7" t="n">
-        <v>0.2931065832368425</v>
+        <v>0.2950433509063108</v>
       </c>
       <c r="CB7" t="n">
-        <v>0.7710475966803008</v>
+        <v>0.7587073562732791</v>
       </c>
       <c r="CC7" t="n">
-        <v>0.5329139541191898</v>
+        <v>0.5288921444778456</v>
       </c>
       <c r="CD7" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -2364,244 +2364,244 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9119733200383611</v>
+        <v>0.920299683837225</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8549567618360945</v>
+        <v>0.8665856639970623</v>
       </c>
       <c r="E8" t="n">
-        <v>102.5366037881779</v>
+        <v>103.1798150245895</v>
       </c>
       <c r="F8" t="n">
-        <v>96.41097510705598</v>
+        <v>97.49448698844297</v>
       </c>
       <c r="G8" t="n">
-        <v>6.125628681121966</v>
+        <v>5.685328036146511</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2921885835132531</v>
+        <v>0.2910332453567848</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7226619977721135</v>
+        <v>0.7233232245346598</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5127543975734881</v>
+        <v>0.5124566797008566</v>
       </c>
       <c r="K8" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L8" t="n">
-        <v>1953</v>
+        <v>1739</v>
       </c>
       <c r="M8" t="n">
-        <v>447</v>
+        <v>402</v>
       </c>
       <c r="N8" t="n">
-        <v>879</v>
+        <v>783</v>
       </c>
       <c r="O8" t="n">
+        <v>199</v>
+      </c>
+      <c r="P8" t="n">
+        <v>614</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>338</v>
+      </c>
+      <c r="R8" t="n">
+        <v>436</v>
+      </c>
+      <c r="S8" t="n">
+        <v>207</v>
+      </c>
+      <c r="T8" t="n">
+        <v>550</v>
+      </c>
+      <c r="U8" t="n">
+        <v>272</v>
+      </c>
+      <c r="V8" t="n">
+        <v>176</v>
+      </c>
+      <c r="W8" t="n">
+        <v>303</v>
+      </c>
+      <c r="X8" t="n">
+        <v>522</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>437</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>41</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>1664</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1891.84</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1684.84</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>2225</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>212</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>379</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>94</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>288</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>161</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>213</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>93</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>254</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>153</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>88</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>148</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>260</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>212</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>908.72</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>815.72</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0.9528635639893417</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.8768305795184663</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>106.2192798779225</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>102.2300908293326</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>3.989189048589867</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0.291936799470835</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0.652794185460415</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0.4856462798534153</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>190</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>404</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>105</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>326</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>177</v>
+      </c>
+      <c r="BK8" t="n">
         <v>223</v>
       </c>
-      <c r="P8" t="n">
-        <v>694</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>390</v>
-      </c>
-      <c r="R8" t="n">
-        <v>515</v>
-      </c>
-      <c r="S8" t="n">
-        <v>240</v>
-      </c>
-      <c r="T8" t="n">
-        <v>632</v>
-      </c>
-      <c r="U8" t="n">
-        <v>305</v>
-      </c>
-      <c r="V8" t="n">
-        <v>195</v>
-      </c>
-      <c r="W8" t="n">
-        <v>345</v>
-      </c>
-      <c r="X8" t="n">
-        <v>588</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>501</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>47</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>1857</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>2144.6</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>1904.6</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>26</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>2625</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>243</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>437</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>112</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>347</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>195</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>266</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>116</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>310</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>180</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>102</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>174</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>306</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>253</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>26</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>1075.04</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>959.04</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>0.9450396025167976</v>
-      </c>
-      <c r="AW8" t="n">
-        <v>0.8541308489293147</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>105.9617102748234</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>99.84877886962407</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>6.112931405199306</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>0.2945176182002636</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>0.6554626013724879</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>0.4884543345648257</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>13</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>2600</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>204</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>442</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>111</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>347</v>
-      </c>
-      <c r="BJ8" t="n">
-        <v>195</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>249</v>
-      </c>
       <c r="BL8" t="n">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="BM8" t="n">
-        <v>322</v>
+        <v>296</v>
       </c>
       <c r="BN8" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="BO8" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="BP8" t="n">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="BQ8" t="n">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="BR8" t="n">
-        <v>248</v>
+        <v>225</v>
       </c>
       <c r="BS8" t="n">
         <v>21</v>
       </c>
       <c r="BT8" t="n">
-        <v>1069.56</v>
+        <v>983.12</v>
       </c>
       <c r="BU8" t="n">
-        <v>945.5600000000001</v>
+        <v>869.12</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.8789070375599244</v>
+        <v>0.8904494603644514</v>
       </c>
       <c r="BW8" t="n">
-        <v>0.8557826747428751</v>
+        <v>0.857194491435776</v>
       </c>
       <c r="BX8" t="n">
-        <v>99.11149730153252</v>
+        <v>100.3936389090342</v>
       </c>
       <c r="BY8" t="n">
-        <v>92.97317134448791</v>
+        <v>93.15351680096079</v>
       </c>
       <c r="BZ8" t="n">
-        <v>6.138325957044628</v>
+        <v>7.24012210807344</v>
       </c>
       <c r="CA8" t="n">
-        <v>0.2898595488262426</v>
+        <v>0.2902049874189057</v>
       </c>
       <c r="CB8" t="n">
-        <v>0.789861394171739</v>
+        <v>0.7879748436860505</v>
       </c>
       <c r="CC8" t="n">
-        <v>0.5370544605821501</v>
+        <v>0.537032879561011</v>
       </c>
       <c r="CD8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -2616,244 +2616,244 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9074383019965062</v>
+        <v>0.9075496641151679</v>
       </c>
       <c r="D9" t="n">
-        <v>0.941941356293193</v>
+        <v>0.9377677938645381</v>
       </c>
       <c r="E9" t="n">
-        <v>103.1985382651584</v>
+        <v>102.7577502704969</v>
       </c>
       <c r="F9" t="n">
-        <v>105.7893439291211</v>
+        <v>105.3563154872195</v>
       </c>
       <c r="G9" t="n">
-        <v>-2.5908056639628</v>
+        <v>-2.598565216722719</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3022579933117567</v>
+        <v>0.2903266752263259</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7028285153202911</v>
+        <v>0.7023892023799054</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4943156367299719</v>
+        <v>0.4872716391176588</v>
       </c>
       <c r="K9" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L9" t="n">
-        <v>2143</v>
+        <v>1887</v>
       </c>
       <c r="M9" t="n">
-        <v>576</v>
+        <v>493</v>
       </c>
       <c r="N9" t="n">
-        <v>1192</v>
+        <v>1032</v>
       </c>
       <c r="O9" t="n">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="P9" t="n">
-        <v>611</v>
+        <v>550</v>
       </c>
       <c r="Q9" t="n">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="R9" t="n">
-        <v>560</v>
+        <v>516</v>
       </c>
       <c r="S9" t="n">
-        <v>288</v>
+        <v>244</v>
       </c>
       <c r="T9" t="n">
-        <v>611</v>
+        <v>541</v>
       </c>
       <c r="U9" t="n">
-        <v>385</v>
+        <v>327</v>
       </c>
       <c r="V9" t="n">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="W9" t="n">
-        <v>320</v>
+        <v>276</v>
       </c>
       <c r="X9" t="n">
-        <v>593</v>
+        <v>523</v>
       </c>
       <c r="Y9" t="n">
-        <v>545</v>
+        <v>491</v>
       </c>
       <c r="Z9" t="n">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="AA9" t="n">
-        <v>2208</v>
+        <v>1951</v>
       </c>
       <c r="AB9" t="n">
-        <v>2369.4</v>
+        <v>2085.04</v>
       </c>
       <c r="AC9" t="n">
-        <v>2081.4</v>
+        <v>1841.04</v>
       </c>
       <c r="AD9" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE9" t="n">
-        <v>2600</v>
+        <v>2400</v>
       </c>
       <c r="AF9" t="n">
+        <v>228</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>525</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>88</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>281</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>190</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>267</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>117</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>287</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>130</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>79</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>146</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>279</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>252</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>34</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>1069.48</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>952.48</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.8545783368381131</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.8977498791297335</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>95.95352995678292</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>101.9072785225854</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>-5.953748565802472</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.2604700854700854</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>0.6910843968682544</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.4639699831447001</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>265</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>507</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>90</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>269</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>177</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>249</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>127</v>
+      </c>
+      <c r="BM9" t="n">
         <v>254</v>
       </c>
-      <c r="AG9" t="n">
-        <v>570</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>96</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>305</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>199</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>284</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>133</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>316</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>148</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>91</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>168</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>301</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>269</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>38</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>1167.96</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>1034.96</v>
-      </c>
-      <c r="AV9" t="n">
-        <v>0.8552353428590019</v>
-      </c>
-      <c r="AW9" t="n">
-        <v>0.8877269376608032</v>
-      </c>
-      <c r="AX9" t="n">
-        <v>96.499818893182</v>
-      </c>
-      <c r="AY9" t="n">
-        <v>100.6652784974241</v>
-      </c>
-      <c r="AZ9" t="n">
-        <v>-4.165459604242114</v>
-      </c>
-      <c r="BA9" t="n">
-        <v>0.2766330200719341</v>
-      </c>
-      <c r="BB9" t="n">
-        <v>0.6951232696929844</v>
-      </c>
-      <c r="BC9" t="n">
-        <v>0.4756983195308296</v>
-      </c>
-      <c r="BD9" t="n">
-        <v>13</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>2625</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>322</v>
-      </c>
-      <c r="BG9" t="n">
-        <v>622</v>
-      </c>
-      <c r="BH9" t="n">
-        <v>103</v>
-      </c>
-      <c r="BI9" t="n">
-        <v>306</v>
-      </c>
-      <c r="BJ9" t="n">
-        <v>195</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>276</v>
-      </c>
-      <c r="BL9" t="n">
-        <v>155</v>
-      </c>
-      <c r="BM9" t="n">
-        <v>295</v>
-      </c>
       <c r="BN9" t="n">
-        <v>237</v>
+        <v>197</v>
       </c>
       <c r="BO9" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="BP9" t="n">
-        <v>152</v>
+        <v>130</v>
       </c>
       <c r="BQ9" t="n">
-        <v>292</v>
+        <v>244</v>
       </c>
       <c r="BR9" t="n">
-        <v>276</v>
+        <v>239</v>
       </c>
       <c r="BS9" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="BT9" t="n">
-        <v>1201.44</v>
+        <v>1015.56</v>
       </c>
       <c r="BU9" t="n">
-        <v>1046.44</v>
+        <v>888.5599999999999</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.9596412611340105</v>
+        <v>0.9653365665992278</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.9961557749255829</v>
+        <v>0.9814237008479616</v>
       </c>
       <c r="BX9" t="n">
-        <v>109.8972576371348</v>
+        <v>110.1805360672757</v>
       </c>
       <c r="BY9" t="n">
-        <v>110.9134093608183</v>
+        <v>109.1189012668205</v>
       </c>
       <c r="BZ9" t="n">
-        <v>-1.016151723683486</v>
+        <v>1.061634800455194</v>
       </c>
       <c r="CA9" t="n">
-        <v>0.3278829665515792</v>
+        <v>0.3228975004149517</v>
       </c>
       <c r="CB9" t="n">
-        <v>0.710533760947598</v>
+        <v>0.7147217174835249</v>
       </c>
       <c r="CC9" t="n">
-        <v>0.5129329539291143</v>
+        <v>0.5126916274517955</v>
       </c>
       <c r="CD9" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -2868,244 +2868,244 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8626835083455197</v>
+        <v>0.8744942934739314</v>
       </c>
       <c r="D10" t="n">
-        <v>0.954735246464515</v>
+        <v>0.9594853166524682</v>
       </c>
       <c r="E10" t="n">
-        <v>96.52980328468763</v>
+        <v>97.71766420054797</v>
       </c>
       <c r="F10" t="n">
-        <v>108.8989524643081</v>
+        <v>109.4609479895273</v>
       </c>
       <c r="G10" t="n">
-        <v>-12.36914917962046</v>
+        <v>-11.74328378897937</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2542061146288713</v>
+        <v>0.2527133992782546</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6813417670296675</v>
+        <v>0.6838153734708773</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4648134220734654</v>
+        <v>0.4664312710671646</v>
       </c>
       <c r="K10" t="n">
-        <v>5200</v>
+        <v>4600</v>
       </c>
       <c r="L10" t="n">
-        <v>1984</v>
+        <v>1776</v>
       </c>
       <c r="M10" t="n">
-        <v>528</v>
+        <v>472</v>
       </c>
       <c r="N10" t="n">
-        <v>1130</v>
+        <v>1004</v>
       </c>
       <c r="O10" t="n">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="P10" t="n">
-        <v>608</v>
+        <v>539</v>
       </c>
       <c r="Q10" t="n">
-        <v>349</v>
+        <v>316</v>
       </c>
       <c r="R10" t="n">
-        <v>508</v>
+        <v>455</v>
       </c>
       <c r="S10" t="n">
-        <v>242</v>
+        <v>212</v>
       </c>
       <c r="T10" t="n">
-        <v>615</v>
+        <v>549</v>
       </c>
       <c r="U10" t="n">
-        <v>338</v>
+        <v>299</v>
       </c>
       <c r="V10" t="n">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="W10" t="n">
-        <v>337</v>
+        <v>287</v>
       </c>
       <c r="X10" t="n">
-        <v>504</v>
+        <v>454</v>
       </c>
       <c r="Y10" t="n">
-        <v>515</v>
+        <v>457</v>
       </c>
       <c r="Z10" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="AA10" t="n">
-        <v>2231</v>
+        <v>1980</v>
       </c>
       <c r="AB10" t="n">
-        <v>2298.52</v>
+        <v>2030.2</v>
       </c>
       <c r="AC10" t="n">
-        <v>2056.52</v>
+        <v>1818.2</v>
       </c>
       <c r="AD10" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>223</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>474</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>77</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>252</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>146</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>215</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>91</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>257</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>133</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>74</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>135</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>218</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>213</v>
+      </c>
+      <c r="AS10" t="n">
         <v>26</v>
       </c>
-      <c r="AE10" t="n">
-        <v>2600</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>258</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>558</v>
-      </c>
-      <c r="AH10" t="n">
-        <v>92</v>
-      </c>
-      <c r="AI10" t="n">
-        <v>297</v>
-      </c>
-      <c r="AJ10" t="n">
+      <c r="AT10" t="n">
+        <v>955.6</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>864.6</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.8607424610437093</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.9538720664164063</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>95.12220108749398</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>110.876619074607</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>-15.75441798711308</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.2324342023665278</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0.6445318535405081</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>0.441621518123105</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>2400</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>249</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>530</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>95</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>287</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>170</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>240</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>121</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>292</v>
+      </c>
+      <c r="BN10" t="n">
         <v>166</v>
       </c>
-      <c r="AK10" t="n">
-        <v>245</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>111</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>305</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>160</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>93</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>166</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>251</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>249</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>30</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>1128.8</v>
-      </c>
-      <c r="AU10" t="n">
-        <v>1017.8</v>
-      </c>
-      <c r="AV10" t="n">
-        <v>0.8474706075792502</v>
-      </c>
-      <c r="AW10" t="n">
-        <v>0.9526482646570322</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>94.06550327355535</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>110.0275756925837</v>
-      </c>
-      <c r="AZ10" t="n">
-        <v>-15.96207241902832</v>
-      </c>
-      <c r="BA10" t="n">
-        <v>0.2382551358901805</v>
-      </c>
-      <c r="BB10" t="n">
-        <v>0.6575054597831449</v>
-      </c>
-      <c r="BC10" t="n">
-        <v>0.4485772919141426</v>
-      </c>
-      <c r="BD10" t="n">
-        <v>13</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>2600</v>
-      </c>
-      <c r="BF10" t="n">
-        <v>270</v>
-      </c>
-      <c r="BG10" t="n">
-        <v>572</v>
-      </c>
-      <c r="BH10" t="n">
-        <v>101</v>
-      </c>
-      <c r="BI10" t="n">
-        <v>311</v>
-      </c>
-      <c r="BJ10" t="n">
-        <v>183</v>
-      </c>
-      <c r="BK10" t="n">
-        <v>263</v>
-      </c>
-      <c r="BL10" t="n">
-        <v>131</v>
-      </c>
-      <c r="BM10" t="n">
-        <v>310</v>
-      </c>
-      <c r="BN10" t="n">
-        <v>178</v>
-      </c>
       <c r="BO10" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="BP10" t="n">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="BQ10" t="n">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="BR10" t="n">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="BS10" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="BT10" t="n">
-        <v>1169.72</v>
+        <v>1074.6</v>
       </c>
       <c r="BU10" t="n">
-        <v>1038.72</v>
+        <v>953.6</v>
       </c>
       <c r="BV10" t="n">
-        <v>0.8778964091117891</v>
+        <v>0.8871001398683015</v>
       </c>
       <c r="BW10" t="n">
-        <v>0.9568222282719974</v>
+        <v>0.9646307960355248</v>
       </c>
       <c r="BX10" t="n">
-        <v>98.9941032958199</v>
+        <v>100.0968387208475</v>
       </c>
       <c r="BY10" t="n">
-        <v>107.7703292360325</v>
+        <v>108.163249494871</v>
       </c>
       <c r="BZ10" t="n">
-        <v>-8.776225940212594</v>
+        <v>-8.066410774023462</v>
       </c>
       <c r="CA10" t="n">
-        <v>0.270157093367562</v>
+        <v>0.2713026631140041</v>
       </c>
       <c r="CB10" t="n">
-        <v>0.7051780742761899</v>
+        <v>0.7198252667403823</v>
       </c>
       <c r="CC10" t="n">
-        <v>0.4810495522327883</v>
+        <v>0.4891735445992193</v>
       </c>
       <c r="CD10" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -3120,244 +3120,244 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.9299857744533923</v>
+        <v>0.9289725456965839</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8885359875803521</v>
+        <v>0.8776559951518826</v>
       </c>
       <c r="E11" t="n">
-        <v>107.530833419519</v>
+        <v>107.5114468186898</v>
       </c>
       <c r="F11" t="n">
-        <v>99.48521802113757</v>
+        <v>98.37252349834807</v>
       </c>
       <c r="G11" t="n">
-        <v>8.045615398381431</v>
+        <v>9.138923320341783</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3393090582068566</v>
+        <v>0.3404855387798324</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7203757533109829</v>
+        <v>0.7190976862161299</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5213055346005016</v>
+        <v>0.5219018030636192</v>
       </c>
       <c r="K11" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L11" t="n">
-        <v>2096</v>
+        <v>1863</v>
       </c>
       <c r="M11" t="n">
+        <v>470</v>
+      </c>
+      <c r="N11" t="n">
+        <v>955</v>
+      </c>
+      <c r="O11" t="n">
+        <v>196</v>
+      </c>
+      <c r="P11" t="n">
+        <v>597</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>335</v>
+      </c>
+      <c r="R11" t="n">
+        <v>459</v>
+      </c>
+      <c r="S11" t="n">
+        <v>276</v>
+      </c>
+      <c r="T11" t="n">
         <v>529</v>
       </c>
-      <c r="N11" t="n">
-        <v>1066</v>
-      </c>
-      <c r="O11" t="n">
-        <v>222</v>
-      </c>
-      <c r="P11" t="n">
-        <v>681</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>372</v>
-      </c>
-      <c r="R11" t="n">
-        <v>507</v>
-      </c>
-      <c r="S11" t="n">
-        <v>308</v>
-      </c>
-      <c r="T11" t="n">
-        <v>591</v>
-      </c>
       <c r="U11" t="n">
-        <v>373</v>
+        <v>329</v>
       </c>
       <c r="V11" t="n">
-        <v>197</v>
+        <v>177</v>
       </c>
       <c r="W11" t="n">
-        <v>284</v>
+        <v>252</v>
       </c>
       <c r="X11" t="n">
-        <v>521</v>
+        <v>468</v>
       </c>
       <c r="Y11" t="n">
-        <v>510</v>
+        <v>449</v>
       </c>
       <c r="Z11" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="AA11" t="n">
-        <v>1896</v>
+        <v>1672</v>
       </c>
       <c r="AB11" t="n">
-        <v>2254.08</v>
+        <v>2005.96</v>
       </c>
       <c r="AC11" t="n">
-        <v>1946.08</v>
+        <v>1729.96</v>
       </c>
       <c r="AD11" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE11" t="n">
-        <v>2625</v>
+        <v>2425</v>
       </c>
       <c r="AF11" t="n">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="AG11" t="n">
-        <v>513</v>
+        <v>473</v>
       </c>
       <c r="AH11" t="n">
+        <v>107</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>310</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>192</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>249</v>
+      </c>
+      <c r="AL11" t="n">
         <v>116</v>
       </c>
-      <c r="AI11" t="n">
-        <v>335</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>199</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>256</v>
-      </c>
-      <c r="AL11" t="n">
+      <c r="AM11" t="n">
+        <v>279</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>152</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>82</v>
+      </c>
+      <c r="AP11" t="n">
         <v>127</v>
       </c>
-      <c r="AM11" t="n">
-        <v>300</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>170</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>87</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>137</v>
-      </c>
       <c r="AQ11" t="n">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="AR11" t="n">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="AS11" t="n">
         <v>28</v>
       </c>
       <c r="AT11" t="n">
-        <v>1097.64</v>
+        <v>1019.56</v>
       </c>
       <c r="AU11" t="n">
-        <v>970.64</v>
+        <v>903.5600000000001</v>
       </c>
       <c r="AV11" t="n">
-        <v>0.9549941636036562</v>
+        <v>0.9598673111170756</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.8876934526951217</v>
+        <v>0.8869492010385619</v>
       </c>
       <c r="AX11" t="n">
-        <v>107.9032368005818</v>
+        <v>108.1990889231507</v>
       </c>
       <c r="AY11" t="n">
-        <v>100.8125104977241</v>
+        <v>100.6068296694158</v>
       </c>
       <c r="AZ11" t="n">
-        <v>7.090726302857669</v>
+        <v>7.592259253734852</v>
       </c>
       <c r="BA11" t="n">
-        <v>0.2886440357897871</v>
+        <v>0.2857369211252105</v>
       </c>
       <c r="BB11" t="n">
-        <v>0.6924523604415203</v>
+        <v>0.6937051109084211</v>
       </c>
       <c r="BC11" t="n">
-        <v>0.4889409826508734</v>
+        <v>0.4886604235128051</v>
       </c>
       <c r="BD11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BE11" t="n">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="BF11" t="n">
-        <v>278</v>
+        <v>237</v>
       </c>
       <c r="BG11" t="n">
-        <v>553</v>
+        <v>482</v>
       </c>
       <c r="BH11" t="n">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="BI11" t="n">
-        <v>346</v>
+        <v>287</v>
       </c>
       <c r="BJ11" t="n">
-        <v>173</v>
+        <v>143</v>
       </c>
       <c r="BK11" t="n">
-        <v>251</v>
+        <v>210</v>
       </c>
       <c r="BL11" t="n">
-        <v>181</v>
+        <v>160</v>
       </c>
       <c r="BM11" t="n">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="BN11" t="n">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="BO11" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="BP11" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="BQ11" t="n">
-        <v>247</v>
+        <v>210</v>
       </c>
       <c r="BR11" t="n">
-        <v>261</v>
+        <v>216</v>
       </c>
       <c r="BS11" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="BT11" t="n">
-        <v>1156.44</v>
+        <v>986.4</v>
       </c>
       <c r="BU11" t="n">
-        <v>975.4400000000001</v>
+        <v>826.4</v>
       </c>
       <c r="BV11" t="n">
-        <v>0.9049773853031284</v>
+        <v>0.8952691652378657</v>
       </c>
       <c r="BW11" t="n">
-        <v>0.8893785224655826</v>
+        <v>0.8675179523664145</v>
       </c>
       <c r="BX11" t="n">
-        <v>107.1584300384561</v>
+        <v>106.7612917956417</v>
       </c>
       <c r="BY11" t="n">
-        <v>98.15792554455093</v>
+        <v>95.93509858445594</v>
       </c>
       <c r="BZ11" t="n">
-        <v>9.00050449390519</v>
+        <v>10.82619321118571</v>
       </c>
       <c r="CA11" t="n">
-        <v>0.3899740806239261</v>
+        <v>0.4002113034939654</v>
       </c>
       <c r="CB11" t="n">
-        <v>0.7482991461804459</v>
+        <v>0.7467986774609031</v>
       </c>
       <c r="CC11" t="n">
-        <v>0.5536700865501298</v>
+        <v>0.5581651262099621</v>
       </c>
       <c r="CD11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -3372,244 +3372,244 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.8248385152699362</v>
+        <v>0.8122301987716145</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9410935140754079</v>
+        <v>0.9287289346349934</v>
       </c>
       <c r="E12" t="n">
-        <v>94.03142468862585</v>
+        <v>92.48775168337444</v>
       </c>
       <c r="F12" t="n">
-        <v>107.5033439679326</v>
+        <v>106.2670643679404</v>
       </c>
       <c r="G12" t="n">
-        <v>-13.47191927930673</v>
+        <v>-13.77931268456595</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2884786274367068</v>
+        <v>0.2863344237243753</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6639515001162397</v>
+        <v>0.6696014887442377</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4656106154623132</v>
+        <v>0.4690729023434713</v>
       </c>
       <c r="K12" t="n">
-        <v>5225</v>
+        <v>4625</v>
       </c>
       <c r="L12" t="n">
-        <v>1927</v>
+        <v>1699</v>
       </c>
       <c r="M12" t="n">
-        <v>441</v>
+        <v>397</v>
       </c>
       <c r="N12" t="n">
-        <v>943</v>
+        <v>841</v>
       </c>
       <c r="O12" t="n">
-        <v>231</v>
+        <v>198</v>
       </c>
       <c r="P12" t="n">
-        <v>795</v>
+        <v>710</v>
       </c>
       <c r="Q12" t="n">
-        <v>352</v>
+        <v>311</v>
       </c>
       <c r="R12" t="n">
-        <v>563</v>
+        <v>506</v>
       </c>
       <c r="S12" t="n">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="T12" t="n">
-        <v>579</v>
+        <v>530</v>
       </c>
       <c r="U12" t="n">
-        <v>302</v>
+        <v>263</v>
       </c>
       <c r="V12" t="n">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="W12" t="n">
-        <v>353</v>
+        <v>318</v>
       </c>
       <c r="X12" t="n">
-        <v>585</v>
+        <v>512</v>
       </c>
       <c r="Y12" t="n">
-        <v>534</v>
+        <v>474</v>
       </c>
       <c r="Z12" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="AA12" t="n">
-        <v>2163</v>
+        <v>1901</v>
       </c>
       <c r="AB12" t="n">
-        <v>2338.72</v>
+        <v>2091.64</v>
       </c>
       <c r="AC12" t="n">
-        <v>2051.72</v>
+        <v>1836.64</v>
       </c>
       <c r="AD12" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE12" t="n">
-        <v>2625</v>
+        <v>2425</v>
       </c>
       <c r="AF12" t="n">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="AG12" t="n">
-        <v>470</v>
+        <v>433</v>
       </c>
       <c r="AH12" t="n">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="AI12" t="n">
-        <v>388</v>
+        <v>363</v>
       </c>
       <c r="AJ12" t="n">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="AK12" t="n">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="AL12" t="n">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="AM12" t="n">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="AN12" t="n">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="AO12" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="AP12" t="n">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AQ12" t="n">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="AR12" t="n">
-        <v>264</v>
+        <v>243</v>
       </c>
       <c r="AS12" t="n">
         <v>10</v>
       </c>
       <c r="AT12" t="n">
-        <v>1171.8</v>
+        <v>1092.2</v>
       </c>
       <c r="AU12" t="n">
-        <v>1026.8</v>
+        <v>957.2</v>
       </c>
       <c r="AV12" t="n">
-        <v>0.7895109001593842</v>
+        <v>0.780973491923085</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.9504660006176285</v>
+        <v>0.9246813820920226</v>
       </c>
       <c r="AX12" t="n">
-        <v>89.98913894325027</v>
+        <v>88.98727600078165</v>
       </c>
       <c r="AY12" t="n">
-        <v>108.4683935852594</v>
+        <v>105.8572070857854</v>
       </c>
       <c r="AZ12" t="n">
-        <v>-18.47925464200912</v>
+        <v>-16.86993108500374</v>
       </c>
       <c r="BA12" t="n">
-        <v>0.285603484750889</v>
+        <v>0.2862556269986483</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.6653005916939259</v>
+        <v>0.6691550060811181</v>
       </c>
       <c r="BC12" t="n">
-        <v>0.4642517722155883</v>
+        <v>0.4693136889060686</v>
       </c>
       <c r="BD12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="BE12" t="n">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="BF12" t="n">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="BG12" t="n">
-        <v>473</v>
+        <v>408</v>
       </c>
       <c r="BH12" t="n">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="BI12" t="n">
-        <v>407</v>
+        <v>347</v>
       </c>
       <c r="BJ12" t="n">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="BK12" t="n">
-        <v>293</v>
+        <v>251</v>
       </c>
       <c r="BL12" t="n">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="BM12" t="n">
-        <v>286</v>
+        <v>250</v>
       </c>
       <c r="BN12" t="n">
-        <v>159</v>
+        <v>129</v>
       </c>
       <c r="BO12" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="BP12" t="n">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="BQ12" t="n">
-        <v>302</v>
+        <v>240</v>
       </c>
       <c r="BR12" t="n">
-        <v>270</v>
+        <v>231</v>
       </c>
       <c r="BS12" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="BT12" t="n">
-        <v>1166.92</v>
+        <v>999.4399999999999</v>
       </c>
       <c r="BU12" t="n">
-        <v>1024.92</v>
+        <v>879.4399999999999</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.8601661303804882</v>
+        <v>0.8463284244245558</v>
       </c>
       <c r="BW12" t="n">
-        <v>0.9317210275331868</v>
+        <v>0.9331444465000523</v>
       </c>
       <c r="BX12" t="n">
-        <v>98.07371043400144</v>
+        <v>96.30645242802116</v>
       </c>
       <c r="BY12" t="n">
-        <v>106.5382943506058</v>
+        <v>106.7141814030186</v>
       </c>
       <c r="BZ12" t="n">
-        <v>-8.464583916604328</v>
+        <v>-10.40772897499745</v>
       </c>
       <c r="CA12" t="n">
-        <v>0.2913537701225246</v>
+        <v>0.2864203837888049</v>
       </c>
       <c r="CB12" t="n">
-        <v>0.6626024085385537</v>
+        <v>0.6700885607403687</v>
       </c>
       <c r="CC12" t="n">
-        <v>0.4669694587090379</v>
+        <v>0.4688102260933651</v>
       </c>
       <c r="CD12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -3624,244 +3624,244 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.8676693989873457</v>
+        <v>0.8662516168041164</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8927669910258835</v>
+        <v>0.8867779119028539</v>
       </c>
       <c r="E13" t="n">
-        <v>98.4164528127381</v>
+        <v>98.48572698935251</v>
       </c>
       <c r="F13" t="n">
-        <v>102.627499514625</v>
+        <v>102.1776950380084</v>
       </c>
       <c r="G13" t="n">
-        <v>-4.211046701886889</v>
+        <v>-3.691968048655815</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2950322612221828</v>
+        <v>0.2951416585484984</v>
       </c>
       <c r="I13" t="n">
-        <v>0.6819897594025529</v>
+        <v>0.6778591353754232</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4926680829634689</v>
+        <v>0.489465059472887</v>
       </c>
       <c r="K13" t="n">
-        <v>5250</v>
+        <v>4625</v>
       </c>
       <c r="L13" t="n">
-        <v>1897</v>
+        <v>1676</v>
       </c>
       <c r="M13" t="n">
-        <v>424</v>
+        <v>376</v>
       </c>
       <c r="N13" t="n">
-        <v>905</v>
+        <v>809</v>
       </c>
       <c r="O13" t="n">
-        <v>212</v>
+        <v>184</v>
       </c>
       <c r="P13" t="n">
-        <v>687</v>
+        <v>608</v>
       </c>
       <c r="Q13" t="n">
-        <v>413</v>
+        <v>372</v>
       </c>
       <c r="R13" t="n">
-        <v>569</v>
+        <v>507</v>
       </c>
       <c r="S13" t="n">
-        <v>261</v>
+        <v>235</v>
       </c>
       <c r="T13" t="n">
-        <v>629</v>
+        <v>560</v>
       </c>
       <c r="U13" t="n">
-        <v>349</v>
+        <v>305</v>
       </c>
       <c r="V13" t="n">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="W13" t="n">
-        <v>348</v>
+        <v>298</v>
       </c>
       <c r="X13" t="n">
-        <v>505</v>
+        <v>444</v>
       </c>
       <c r="Y13" t="n">
-        <v>564</v>
+        <v>497</v>
       </c>
       <c r="Z13" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AA13" t="n">
-        <v>1997</v>
+        <v>1768</v>
       </c>
       <c r="AB13" t="n">
-        <v>2190.36</v>
+        <v>1938.08</v>
       </c>
       <c r="AC13" t="n">
-        <v>1929.36</v>
+        <v>1703.08</v>
       </c>
       <c r="AD13" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE13" t="n">
-        <v>2625</v>
+        <v>2200</v>
       </c>
       <c r="AF13" t="n">
-        <v>208</v>
+        <v>180</v>
       </c>
       <c r="AG13" t="n">
-        <v>438</v>
+        <v>379</v>
       </c>
       <c r="AH13" t="n">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="AI13" t="n">
-        <v>362</v>
+        <v>307</v>
       </c>
       <c r="AJ13" t="n">
-        <v>191</v>
+        <v>157</v>
       </c>
       <c r="AK13" t="n">
-        <v>267</v>
+        <v>216</v>
       </c>
       <c r="AL13" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="AM13" t="n">
-        <v>320</v>
+        <v>274</v>
       </c>
       <c r="AN13" t="n">
-        <v>171</v>
+        <v>142</v>
       </c>
       <c r="AO13" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="AP13" t="n">
-        <v>181</v>
+        <v>141</v>
       </c>
       <c r="AQ13" t="n">
-        <v>264</v>
+        <v>219</v>
       </c>
       <c r="AR13" t="n">
-        <v>285</v>
+        <v>234</v>
       </c>
       <c r="AS13" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="AT13" t="n">
-        <v>1098.48</v>
+        <v>922.04</v>
       </c>
       <c r="AU13" t="n">
-        <v>978.48</v>
+        <v>818.04</v>
       </c>
       <c r="AV13" t="n">
-        <v>0.8863501025035112</v>
+        <v>0.8894144198130159</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.8945709986506863</v>
+        <v>0.8827172348176556</v>
       </c>
       <c r="AX13" t="n">
-        <v>99.47793822934469</v>
+        <v>100.257984094802</v>
       </c>
       <c r="AY13" t="n">
-        <v>104.0746868024015</v>
+        <v>103.5541762049924</v>
       </c>
       <c r="AZ13" t="n">
-        <v>-4.596748573056781</v>
+        <v>-3.296192110190386</v>
       </c>
       <c r="BA13" t="n">
-        <v>0.2774695251973814</v>
+        <v>0.2770094388696326</v>
       </c>
       <c r="BB13" t="n">
-        <v>0.6646101887315449</v>
+        <v>0.6523117646285213</v>
       </c>
       <c r="BC13" t="n">
-        <v>0.4828233421570547</v>
+        <v>0.4757019969600209</v>
       </c>
       <c r="BD13" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="BE13" t="n">
-        <v>2625</v>
+        <v>2425</v>
       </c>
       <c r="BF13" t="n">
-        <v>216</v>
+        <v>196</v>
       </c>
       <c r="BG13" t="n">
-        <v>467</v>
+        <v>430</v>
       </c>
       <c r="BH13" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="BI13" t="n">
-        <v>325</v>
+        <v>301</v>
       </c>
       <c r="BJ13" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="BK13" t="n">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="BL13" t="n">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="BM13" t="n">
-        <v>309</v>
+        <v>286</v>
       </c>
       <c r="BN13" t="n">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="BO13" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="BP13" t="n">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="BQ13" t="n">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="BR13" t="n">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="BS13" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="BT13" t="n">
-        <v>1091.88</v>
+        <v>1016.04</v>
       </c>
       <c r="BU13" t="n">
-        <v>950.88</v>
+        <v>885.04</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.8489886954711802</v>
+        <v>0.8450190473792919</v>
       </c>
       <c r="BW13" t="n">
-        <v>0.8909629834010808</v>
+        <v>0.8905001992309524</v>
       </c>
       <c r="BX13" t="n">
-        <v>97.35496739613151</v>
+        <v>96.86115797602379</v>
       </c>
       <c r="BY13" t="n">
-        <v>101.1803122268485</v>
+        <v>100.9159206349396</v>
       </c>
       <c r="BZ13" t="n">
-        <v>-3.825344830716997</v>
+        <v>-4.054762658915791</v>
       </c>
       <c r="CA13" t="n">
-        <v>0.3125949972469843</v>
+        <v>0.3117628599207921</v>
       </c>
       <c r="CB13" t="n">
-        <v>0.6993693300735612</v>
+        <v>0.7012775585600836</v>
       </c>
       <c r="CC13" t="n">
-        <v>0.5025128237698832</v>
+        <v>0.5020812001096812</v>
       </c>
       <c r="CD13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -3876,244 +3876,244 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.8733307571106851</v>
+        <v>0.8680715910960138</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8721105961494597</v>
+        <v>0.8647006698603729</v>
       </c>
       <c r="E14" t="n">
-        <v>101.9781856284093</v>
+        <v>101.551507973791</v>
       </c>
       <c r="F14" t="n">
-        <v>97.32342588109597</v>
+        <v>96.77777159148782</v>
       </c>
       <c r="G14" t="n">
-        <v>4.654759747313313</v>
+        <v>4.77373638230321</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3411425074165455</v>
+        <v>0.3438156591790308</v>
       </c>
       <c r="I14" t="n">
-        <v>0.7381689317935158</v>
+        <v>0.7320050074067112</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5298789081316845</v>
+        <v>0.5287087606466818</v>
       </c>
       <c r="K14" t="n">
-        <v>5200</v>
+        <v>4600</v>
       </c>
       <c r="L14" t="n">
-        <v>2008</v>
+        <v>1762</v>
       </c>
       <c r="M14" t="n">
-        <v>480</v>
+        <v>423</v>
       </c>
       <c r="N14" t="n">
-        <v>923</v>
+        <v>812</v>
       </c>
       <c r="O14" t="n">
-        <v>229</v>
+        <v>197</v>
       </c>
       <c r="P14" t="n">
-        <v>778</v>
+        <v>688</v>
       </c>
       <c r="Q14" t="n">
-        <v>361</v>
+        <v>325</v>
       </c>
       <c r="R14" t="n">
-        <v>566</v>
+        <v>501</v>
       </c>
       <c r="S14" t="n">
-        <v>331</v>
+        <v>295</v>
       </c>
       <c r="T14" t="n">
-        <v>642</v>
+        <v>565</v>
       </c>
       <c r="U14" t="n">
-        <v>404</v>
+        <v>356</v>
       </c>
       <c r="V14" t="n">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="W14" t="n">
-        <v>347</v>
+        <v>307</v>
       </c>
       <c r="X14" t="n">
-        <v>613</v>
+        <v>539</v>
       </c>
       <c r="Y14" t="n">
-        <v>559</v>
+        <v>493</v>
       </c>
       <c r="Z14" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="AA14" t="n">
-        <v>1918</v>
+        <v>1687</v>
       </c>
       <c r="AB14" t="n">
-        <v>2297.04</v>
+        <v>2027.44</v>
       </c>
       <c r="AC14" t="n">
-        <v>1966.04</v>
+        <v>1732.44</v>
       </c>
       <c r="AD14" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AE14" t="n">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="AF14" t="n">
-        <v>233</v>
+        <v>200</v>
       </c>
       <c r="AG14" t="n">
-        <v>459</v>
+        <v>383</v>
       </c>
       <c r="AH14" t="n">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="AI14" t="n">
-        <v>380</v>
+        <v>321</v>
       </c>
       <c r="AJ14" t="n">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="AK14" t="n">
-        <v>286</v>
+        <v>241</v>
       </c>
       <c r="AL14" t="n">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="AM14" t="n">
-        <v>315</v>
+        <v>265</v>
       </c>
       <c r="AN14" t="n">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="AO14" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AP14" t="n">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="AQ14" t="n">
-        <v>311</v>
+        <v>261</v>
       </c>
       <c r="AR14" t="n">
-        <v>285</v>
+        <v>240</v>
       </c>
       <c r="AS14" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="AT14" t="n">
-        <v>1145.84</v>
+        <v>963.04</v>
       </c>
       <c r="AU14" t="n">
-        <v>993.84</v>
+        <v>837.04</v>
       </c>
       <c r="AV14" t="n">
-        <v>0.8618248133053602</v>
+        <v>0.8583665596464773</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.8831482642749321</v>
+        <v>0.8668108248578352</v>
       </c>
       <c r="AX14" t="n">
-        <v>99.40771620235566</v>
+        <v>98.8390228202281</v>
       </c>
       <c r="AY14" t="n">
-        <v>99.95093932277163</v>
+        <v>98.69580460942922</v>
       </c>
       <c r="AZ14" t="n">
-        <v>-0.5432231204159734</v>
+        <v>0.1432182107988702</v>
       </c>
       <c r="BA14" t="n">
-        <v>0.3139699926413749</v>
+        <v>0.3111541068777912</v>
       </c>
       <c r="BB14" t="n">
-        <v>0.7056691577564445</v>
+        <v>0.6941458011580489</v>
       </c>
       <c r="BC14" t="n">
-        <v>0.5029529668341322</v>
+        <v>0.498404046627242</v>
       </c>
       <c r="BD14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="BE14" t="n">
-        <v>2600</v>
+        <v>2400</v>
       </c>
       <c r="BF14" t="n">
-        <v>247</v>
+        <v>223</v>
       </c>
       <c r="BG14" t="n">
-        <v>464</v>
+        <v>429</v>
       </c>
       <c r="BH14" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="BI14" t="n">
-        <v>398</v>
+        <v>367</v>
       </c>
       <c r="BJ14" t="n">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="BK14" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="BL14" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="BM14" t="n">
-        <v>327</v>
+        <v>300</v>
       </c>
       <c r="BN14" t="n">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="BO14" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="BP14" t="n">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="BQ14" t="n">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="BR14" t="n">
-        <v>274</v>
+        <v>253</v>
       </c>
       <c r="BS14" t="n">
         <v>32</v>
       </c>
       <c r="BT14" t="n">
-        <v>1151.2</v>
+        <v>1064.4</v>
       </c>
       <c r="BU14" t="n">
-        <v>972.2</v>
+        <v>895.4</v>
       </c>
       <c r="BV14" t="n">
-        <v>0.8848367009160097</v>
+        <v>0.8769678699247555</v>
       </c>
       <c r="BW14" t="n">
-        <v>0.8610729280239874</v>
+        <v>0.8627663611126991</v>
       </c>
       <c r="BX14" t="n">
-        <v>104.5486550544629</v>
+        <v>104.0379526978904</v>
       </c>
       <c r="BY14" t="n">
-        <v>94.69591243942031</v>
+        <v>95.01957465837485</v>
       </c>
       <c r="BZ14" t="n">
-        <v>9.852742615042599</v>
+        <v>9.018378039515522</v>
       </c>
       <c r="CA14" t="n">
-        <v>0.3683150221917162</v>
+        <v>0.3737554154551673</v>
       </c>
       <c r="CB14" t="n">
-        <v>0.7706687058305876</v>
+        <v>0.7667092798013183</v>
       </c>
       <c r="CC14" t="n">
-        <v>0.556804849429237</v>
+        <v>0.5564880818311684</v>
       </c>
       <c r="CD14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -4128,166 +4128,166 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.9721949559658847</v>
+        <v>0.965344253808349</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8978684965154194</v>
+        <v>0.8745501923131134</v>
       </c>
       <c r="E15" t="n">
-        <v>108.1453418020647</v>
+        <v>107.4757649468014</v>
       </c>
       <c r="F15" t="n">
-        <v>102.5483858884934</v>
+        <v>99.90136847795473</v>
       </c>
       <c r="G15" t="n">
-        <v>5.596955913571333</v>
+        <v>7.574396468846708</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2765476949367658</v>
+        <v>0.2773810386186191</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6874125524246437</v>
+        <v>0.6902649368695861</v>
       </c>
       <c r="J15" t="n">
-        <v>0.4939600241881198</v>
+        <v>0.496353425804429</v>
       </c>
       <c r="K15" t="n">
-        <v>5000</v>
+        <v>4400</v>
       </c>
       <c r="L15" t="n">
-        <v>2138</v>
+        <v>1878</v>
       </c>
       <c r="M15" t="n">
-        <v>539</v>
+        <v>477</v>
       </c>
       <c r="N15" t="n">
-        <v>1004</v>
+        <v>887</v>
       </c>
       <c r="O15" t="n">
-        <v>177</v>
+        <v>155</v>
       </c>
       <c r="P15" t="n">
-        <v>551</v>
+        <v>488</v>
       </c>
       <c r="Q15" t="n">
-        <v>529</v>
+        <v>459</v>
       </c>
       <c r="R15" t="n">
-        <v>729</v>
+        <v>635</v>
       </c>
       <c r="S15" t="n">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="T15" t="n">
-        <v>614</v>
+        <v>548</v>
       </c>
       <c r="U15" t="n">
-        <v>361</v>
+        <v>315</v>
       </c>
       <c r="V15" t="n">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="W15" t="n">
-        <v>328</v>
+        <v>295</v>
       </c>
       <c r="X15" t="n">
-        <v>506</v>
+        <v>433</v>
       </c>
       <c r="Y15" t="n">
-        <v>635</v>
+        <v>556</v>
       </c>
       <c r="Z15" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="AA15" t="n">
-        <v>1999</v>
+        <v>1717</v>
       </c>
       <c r="AB15" t="n">
-        <v>2203.76</v>
+        <v>1949.4</v>
       </c>
       <c r="AC15" t="n">
-        <v>1979.76</v>
+        <v>1749.4</v>
       </c>
       <c r="AD15" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AE15" t="n">
-        <v>2600</v>
+        <v>2000</v>
       </c>
       <c r="AF15" t="n">
-        <v>256</v>
+        <v>194</v>
       </c>
       <c r="AG15" t="n">
-        <v>517</v>
+        <v>400</v>
       </c>
       <c r="AH15" t="n">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="AI15" t="n">
-        <v>282</v>
+        <v>219</v>
       </c>
       <c r="AJ15" t="n">
-        <v>271</v>
+        <v>201</v>
       </c>
       <c r="AK15" t="n">
-        <v>370</v>
+        <v>276</v>
       </c>
       <c r="AL15" t="n">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="AM15" t="n">
-        <v>305</v>
+        <v>239</v>
       </c>
       <c r="AN15" t="n">
-        <v>197</v>
+        <v>151</v>
       </c>
       <c r="AO15" t="n">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="AP15" t="n">
-        <v>171</v>
+        <v>138</v>
       </c>
       <c r="AQ15" t="n">
-        <v>269</v>
+        <v>196</v>
       </c>
       <c r="AR15" t="n">
-        <v>321</v>
+        <v>242</v>
       </c>
       <c r="AS15" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="AT15" t="n">
-        <v>1132.8</v>
+        <v>878.4400000000001</v>
       </c>
       <c r="AU15" t="n">
-        <v>1017.8</v>
+        <v>787.4400000000001</v>
       </c>
       <c r="AV15" t="n">
-        <v>0.942355795608691</v>
+        <v>0.9183325027549543</v>
       </c>
       <c r="AW15" t="n">
-        <v>0.9410171955171721</v>
+        <v>0.9026615359726249</v>
       </c>
       <c r="AX15" t="n">
-        <v>104.7947980596901</v>
+        <v>102.3165658553986</v>
       </c>
       <c r="AY15" t="n">
-        <v>107.9386067846635</v>
+        <v>103.7322347503296</v>
       </c>
       <c r="AZ15" t="n">
-        <v>-3.143808724973396</v>
+        <v>-1.415668894930989</v>
       </c>
       <c r="BA15" t="n">
-        <v>0.2690370633965854</v>
+        <v>0.2686172300346086</v>
       </c>
       <c r="BB15" t="n">
-        <v>0.6723739519422219</v>
+        <v>0.6741376175763685</v>
       </c>
       <c r="BC15" t="n">
-        <v>0.4789968639344391</v>
+        <v>0.4797733994142152</v>
       </c>
       <c r="BD15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="BE15" t="n">
         <v>2400</v>

</xml_diff>